<commit_message>
Drop the populations sheet; derive populations from observations (#26)
Per pearsonca's review: imurun no longer reads a populations sheet. Each
observation now carries its own loc_id/cohort/age/dose (merged into the
observations sheet), and imurun constructs the imuGAP populations from
the observations (one weight-1 row each) via build_populations(). This is
the limited single-row-per-observation flavor of imuGAP's flexibility; a
future version may re-add an optional populations sheet as a pure
expansion.

Updates schema (IMURUN_SCHEMA/IMURUN_SHEETS), the loaders, validate_inputs,
run_fit, the shipped template/example workbooks + test fixtures, and the
make_workbooks generator.
</commit_message>
<xml_diff>
--- a/inst/extdata/imurun_example.xlsx
+++ b/inst/extdata/imurun_example.xlsx
@@ -8,8 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="observations" sheetId="1" r:id="rId1"/>
-    <sheet name="populations" sheetId="2" r:id="rId2"/>
-    <sheet name="locations" sheetId="3" r:id="rId3"/>
+    <sheet name="locations" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -353,7 +352,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -364,10 +363,30 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>loc_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>cohort</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>age</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>positive</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>sample_n</t>
         </is>
@@ -377,132 +396,300 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>61</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Chickadee Elementary</t>
+        </is>
       </c>
       <c r="C2">
-        <v>78</v>
+        <v>4</v>
+      </c>
+      <c r="D2">
+        <v>5</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>16</v>
+      </c>
+      <c r="G2">
+        <v>19</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>72</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Chickadee Elementary</t>
+        </is>
       </c>
       <c r="C3">
-        <v>79</v>
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>14</v>
+      </c>
+      <c r="G3">
+        <v>20</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>69</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Chickadee Elementary</t>
+        </is>
       </c>
       <c r="C4">
-        <v>81</v>
+        <v>6</v>
+      </c>
+      <c r="D4">
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>14</v>
+      </c>
+      <c r="G4">
+        <v>16</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5">
-        <v>68</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Chickadee Elementary</t>
+        </is>
       </c>
       <c r="C5">
-        <v>82</v>
+        <v>7</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>10</v>
+      </c>
+      <c r="G5">
+        <v>13</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6">
-        <v>72</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Chickadee Elementary</t>
+        </is>
       </c>
       <c r="C6">
-        <v>80</v>
+        <v>8</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6">
+        <v>8</v>
+      </c>
+      <c r="G6">
+        <v>13</v>
       </c>
     </row>
     <row r="7">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7">
-        <v>70</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Chickadee Elementary</t>
+        </is>
       </c>
       <c r="C7">
-        <v>83</v>
+        <v>9</v>
+      </c>
+      <c r="D7">
+        <v>5</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="F7">
+        <v>7</v>
+      </c>
+      <c r="G7">
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8">
-        <v>71</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Chickadee Elementary</t>
+        </is>
       </c>
       <c r="C8">
-        <v>82</v>
+        <v>10</v>
+      </c>
+      <c r="D8">
+        <v>5</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
+        <v>6</v>
+      </c>
+      <c r="G8">
+        <v>9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9">
-        <v>69</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Chickadee Elementary</t>
+        </is>
       </c>
       <c r="C9">
-        <v>85</v>
+        <v>11</v>
+      </c>
+      <c r="D9">
+        <v>5</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+      <c r="F9">
+        <v>9</v>
+      </c>
+      <c r="G9">
+        <v>10</v>
       </c>
     </row>
     <row r="10">
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10">
-        <v>83</v>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Chickadee Elementary</t>
+        </is>
       </c>
       <c r="C10">
-        <v>89</v>
+        <v>12</v>
+      </c>
+      <c r="D10">
+        <v>5</v>
+      </c>
+      <c r="E10">
+        <v>2</v>
+      </c>
+      <c r="F10">
+        <v>5</v>
+      </c>
+      <c r="G10">
+        <v>5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11">
-        <v>79</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Chickadee Elementary</t>
+        </is>
       </c>
       <c r="C11">
-        <v>93</v>
+        <v>13</v>
+      </c>
+      <c r="D11">
+        <v>5</v>
+      </c>
+      <c r="E11">
+        <v>2</v>
+      </c>
+      <c r="F11">
+        <v>4</v>
+      </c>
+      <c r="G11">
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12">
-        <v>82</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Chickadee Elementary</t>
+        </is>
       </c>
       <c r="C12">
-        <v>95</v>
+        <v>14</v>
+      </c>
+      <c r="D12">
+        <v>5</v>
+      </c>
+      <c r="E12">
+        <v>2</v>
+      </c>
+      <c r="F12">
+        <v>4</v>
+      </c>
+      <c r="G12">
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13">
-        <v>84</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Chickadee Elementary</t>
+        </is>
       </c>
       <c r="C13">
-        <v>94</v>
+        <v>15</v>
+      </c>
+      <c r="D13">
+        <v>5</v>
+      </c>
+      <c r="E13">
+        <v>2</v>
+      </c>
+      <c r="F13">
+        <v>4</v>
+      </c>
+      <c r="G13">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -512,312 +699,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>obs_id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>loc_id</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>cohort</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>age</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>weight</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Chickadee Elementary</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>4</v>
-      </c>
-      <c r="D2">
-        <v>5</v>
-      </c>
-      <c r="E2">
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Chickadee Elementary</t>
-        </is>
-      </c>
-      <c r="C3">
-        <v>5</v>
-      </c>
-      <c r="D3">
-        <v>5</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Chickadee Elementary</t>
-        </is>
-      </c>
-      <c r="C4">
-        <v>6</v>
-      </c>
-      <c r="D4">
-        <v>5</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Chickadee Elementary</t>
-        </is>
-      </c>
-      <c r="C5">
-        <v>7</v>
-      </c>
-      <c r="D5">
-        <v>5</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Chickadee Elementary</t>
-        </is>
-      </c>
-      <c r="C6">
-        <v>8</v>
-      </c>
-      <c r="D6">
-        <v>5</v>
-      </c>
-      <c r="E6">
-        <v>2</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Chickadee Elementary</t>
-        </is>
-      </c>
-      <c r="C7">
-        <v>9</v>
-      </c>
-      <c r="D7">
-        <v>5</v>
-      </c>
-      <c r="E7">
-        <v>2</v>
-      </c>
-      <c r="F7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Chickadee Elementary</t>
-        </is>
-      </c>
-      <c r="C8">
-        <v>10</v>
-      </c>
-      <c r="D8">
-        <v>5</v>
-      </c>
-      <c r="E8">
-        <v>2</v>
-      </c>
-      <c r="F8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Chickadee Elementary</t>
-        </is>
-      </c>
-      <c r="C9">
-        <v>11</v>
-      </c>
-      <c r="D9">
-        <v>5</v>
-      </c>
-      <c r="E9">
-        <v>2</v>
-      </c>
-      <c r="F9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Chickadee Elementary</t>
-        </is>
-      </c>
-      <c r="C10">
-        <v>12</v>
-      </c>
-      <c r="D10">
-        <v>5</v>
-      </c>
-      <c r="E10">
-        <v>2</v>
-      </c>
-      <c r="F10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Chickadee Elementary</t>
-        </is>
-      </c>
-      <c r="C11">
-        <v>13</v>
-      </c>
-      <c r="D11">
-        <v>5</v>
-      </c>
-      <c r="E11">
-        <v>2</v>
-      </c>
-      <c r="F11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Chickadee Elementary</t>
-        </is>
-      </c>
-      <c r="C12">
-        <v>14</v>
-      </c>
-      <c r="D12">
-        <v>5</v>
-      </c>
-      <c r="E12">
-        <v>2</v>
-      </c>
-      <c r="F12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Chickadee Elementary</t>
-        </is>
-      </c>
-      <c r="C13">
-        <v>15</v>
-      </c>
-      <c r="D13">
-        <v>5</v>
-      </c>
-      <c r="E13">
-        <v>2</v>
-      </c>
-      <c r="F13">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Generate structured .xlsx workbooks with openxlsx2 (#25)
Per @pearsonca: switch the workbook generator from writexl to openxlsx2 so the
shipped template + example carry real spreadsheet structure that makes them
usable for non-technical people:
- an AutoFilter and a frozen header row on each data sheet,
- a Dose dropdown (1/2) via data validation,
- auto-fit column widths,
- a styled (bold, wrapped) instructions tab.

These are cosmetic: the loader reads values with readxl and is blind to
filters / freeze / validation, so parsing is unchanged (full suite still 121
pass). openxlsx2 is used only here at build time -- the shipped .xlsx are
committed -- so it is a dev-only Suggests dependency. The runtime writer
(write_workbook()) stays on writexl, so no new runtime dependency.
</commit_message>
<xml_diff>
--- a/inst/extdata/imurun_example.xlsx
+++ b/inst/extdata/imurun_example.xlsx
@@ -1,38 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView activeTab="0" firstSheet="0" windowHeight="13125" windowWidth="13125" xWindow="0" yWindow="0"/>
   </bookViews>
   <sheets>
-    <sheet name="instructions" sheetId="1" r:id="rId1"/>
-    <sheet name="observations" sheetId="2" r:id="rId2"/>
-    <sheet name="locations" sheetId="3" r:id="rId3"/>
-    <sheet name="target" sheetId="4" r:id="rId4"/>
+    <sheet name="instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="observations" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="locations" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="target" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <b val="1"/>
+      <sz val="13"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
     </font>
   </fonts>
   <fills count="2">
@@ -55,17 +51,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf applyFont="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0"/>
+    <xf applyFont="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
 
@@ -80,44 +79,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -144,14 +143,32 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -178,6 +195,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -189,400 +224,436 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="35000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
+            <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="63000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="40000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A32"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:A31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="100.711"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>instructions</t>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>imurun input workbook -- a beginner-friendly front-end to the imuGAP coverage model.</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>imurun input workbook -- a beginner-friendly front-end to the imuGAP coverage model.</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>This 'instructions' sheet is optional; imurun reads only the data sheets by</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>This 'instructions' sheet is optional; imurun reads only the data sheets by</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>name, so you may delete it. Fill one row per record. You may use these</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>name, so you may delete it. Fill one row per record. You may use these</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>friendly headers or imuGAP's own (loc_id, cohort, ...). Do not add a</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>friendly headers or imuGAP's own (loc_id, cohort, ...). Do not add a</t>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>populations sheet or an observation id -- imurun handles both for you.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>populations sheet or an observation id -- imurun handles both for you.</t>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>observations sheet -- one row per sampled count:</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>observations sheet -- one row per sampled count:</t>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Location          the location (must match a Location in the locations sheet)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Location          the location (must match a Location in the locations sheet)</t>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Birth cohort      positive integer birth-cohort index</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Birth cohort      positive integer birth-cohort index</t>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Age               positive integer age</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Age               positive integer age</t>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Dose              integer dose (1 or 2)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Dose              integer dose (1 or 2)</t>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Vaccinated        number found vaccinated</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Vaccinated        number found vaccinated</t>
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sampled           number sampled (Vaccinated must be &lt;= Sampled)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Sampled           number sampled (Vaccinated must be &lt;= Sampled)</t>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Censored          optional; blank, or 1 for a right-censored observation</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Censored          optional; blank, or 1 for a right-censored observation</t>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>locations sheet -- the location hierarchy:</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>locations sheet -- the location hierarchy:</t>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Location          unique location name</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Location          unique location name</t>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Parent location   the parent's name; leave blank for the single root</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Parent location   the parent's name; leave blank for the single root</t>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>target sheet -- the populations to predict coverage for (required):</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>target sheet -- the populations to predict coverage for (required):</t>
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Location          one or more locations, ';'-separated</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Location          one or more locations, ';'-separated</t>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Birth cohort      reference cohort index for the oldest age in the span</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Birth cohort      reference cohort index for the oldest age in the span</t>
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Youngest age      youngest age to predict</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Youngest age      youngest age to predict</t>
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Oldest age        oldest age to predict</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Oldest age        oldest age to predict</t>
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Dose              optional; blank defaults to the final dose</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Dose              optional; blank defaults to the final dose</t>
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Label             optional; free-text label echoed into the results</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Label             optional; free-text label echoed into the results</t>
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (a Location-only row inherits the cohort/ages/dose from the row above)</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  (a Location-only row inherits the cohort/ages/dose from the row above)</t>
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Validate with:  imurun -h yourfile.xlsx</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Validate with:  imurun -h yourfile.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Fit with:       imurun yourfile.xlsx</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="1" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F699"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="25.711"/>
+    <col min="2" max="2" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+    <col min="3" max="4" bestFit="1" customWidth="1" hidden="false" width="4.711"/>
+    <col min="5" max="5" bestFit="1" customWidth="1" hidden="false" width="10.711"/>
+    <col min="6" max="6" bestFit="1" customWidth="1" hidden="false" width="7.711"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Birth cohort</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Age</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Dose</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Vaccinated</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Sampled</t>
         </is>
@@ -15945,22 +16016,34 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D699">
+      <formula1>"1,2"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <printOptions gridLines="1" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:B29"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="25.711"/>
+    <col min="2" max="2" bestFit="1" customWidth="1" hidden="false" width="15.711"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Parent location</t>
         </is>
@@ -15972,6 +16055,9 @@
           <t>State</t>
         </is>
       </c>
+      <c r="B2" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -16298,42 +16384,52 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <printOptions gridLines="1" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="15.711"/>
+    <col min="2" max="3" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+    <col min="4" max="4" bestFit="1" customWidth="1" hidden="false" width="10.711"/>
+    <col min="5" max="5" bestFit="1" customWidth="1" hidden="false" width="4.711"/>
+    <col min="6" max="6" bestFit="1" customWidth="1" hidden="false" width="17.711"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Birth cohort</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Youngest age</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Oldest age</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Dose</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Label</t>
         </is>
@@ -16369,8 +16465,33 @@
           <t>Watson</t>
         </is>
       </c>
+      <c r="B3" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="C3" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D3" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E3" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E699">
+      <formula1>"1,2"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <printOptions gridLines="1" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Make workbook instructions more hand-holdy; hammer the single-root rule
Per Carl's "more detailed instructions" note. The instructions sheet now:
- leads with a numbered HOW TO USE (fill sheets -> keep headers -> check -> fit),
- spells out that a bad edit fails the check rather than silently producing a
  wrong result, and that extra note columns are ignored,
- rewrites the locations block to emphasize there must be exactly ONE root (the
  single top location with a blank Parent location), every other location names
  its parent, and the chain must reach that root with no loops/second root --
  the degenerate-hierarchy failure behind #24,
- uses plainer wording (whole-number, "how many were ...") throughout.

Regenerated the template, example, and test fixtures. Data unchanged; only the
instructions text differs. All tests pass.
</commit_message>
<xml_diff>
--- a/inst/extdata/imurun_example.xlsx
+++ b/inst/extdata/imurun_example.xlsx
@@ -385,7 +385,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="100.711"/>
@@ -408,203 +408,273 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>This 'instructions' sheet is optional; imurun reads only the data sheets by</t>
+          <t>HOW TO USE THIS FILE</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>name, so you may delete it. Fill one row per record. You may use these</t>
+          <t xml:space="preserve">  1. Fill in the data sheets below (the tabs at the bottom): one row per record.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>friendly headers or imuGAP's own (loc_id, cohort, ...). Do not add a</t>
+          <t xml:space="preserve">  2. Keep the header row on each sheet. You may use these friendly headers or</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>populations sheet or an observation id -- imurun handles both for you.</t>
+          <t xml:space="preserve">     imuGAP's own names (loc_id, cohort, ...); either works.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t xml:space="preserve">  3. Save the file, then check it:   imurun -h yourfile.xlsx</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>observations sheet -- one row per sampled count:</t>
+          <t xml:space="preserve">  4. Fix anything it flags, then fit: imurun yourfile.xlsx</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Location          the location (must match a Location in the locations sheet)</t>
+          <t xml:space="preserve">  A bad edit fails the check with a clear message -- it cannot silently produce a wrong result.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Birth cohort      positive integer birth-cohort index</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Age               positive integer age</t>
+          <t>This 'instructions' sheet is optional: imurun reads only the data sheets by name, so you may</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Dose              integer dose (1 or 2)</t>
+          <t>delete it. Do not add a populations sheet or an observation-id column -- imurun handles both</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Vaccinated        number found vaccinated</t>
+          <t>for you. Extra columns you add for your own notes are ignored.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sampled           number sampled (Vaccinated must be &lt;= Sampled)</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Censored          optional; blank, or 1 for a right-censored observation</t>
+          <t>observations sheet -- one row per sampled count:</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t xml:space="preserve">  Location          the location this count is from (must match a Location in the locations sheet)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>locations sheet -- the location hierarchy:</t>
+          <t xml:space="preserve">  Birth cohort      positive whole-number birth-cohort index</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Location          unique location name</t>
+          <t xml:space="preserve">  Age               positive whole-number age</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Parent location   the parent's name; leave blank for the single root</t>
+          <t xml:space="preserve">  Dose              which dose this count is for: 1 or 2</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t xml:space="preserve">  Vaccinated        how many were found vaccinated</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>target sheet -- the populations to predict coverage for (required):</t>
+          <t xml:space="preserve">  Sampled           how many were sampled (Vaccinated must be &lt;= Sampled)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Location          one or more locations, ';'-separated</t>
+          <t xml:space="preserve">  Censored          optional; leave blank, or put 1 for a right-censored observation</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Birth cohort      reference cohort index for the oldest age in the span</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Youngest age      youngest age to predict</t>
+          <t>locations sheet -- your location hierarchy, written as a tree:</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Oldest age        oldest age to predict</t>
+          <t xml:space="preserve">  Location          a unique name for the location (you choose the names)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Dose              optional; blank defaults to the final dose</t>
+          <t xml:space="preserve">  Parent location   the name of this location's parent (must be another Location in this sheet)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Label             optional; free-text label echoed into the results</t>
+          <t xml:space="preserve">  IMPORTANT: there must be exactly ONE root -- the single top location whose Parent location</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (a Location-only row inherits the cohort/ages/dose from the row above)</t>
+          <t xml:space="preserve">  is left BLANK. Every other location must name its parent, and the parents must chain up to</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t xml:space="preserve">  that one root (no loops, no second root). This is the most common thing to get wrong.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Validate with:  imurun -h yourfile.xlsx</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Fit with:       imurun yourfile.xlsx</t>
+          <t>target sheet -- the populations to predict coverage for (required):</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Location          one or more locations to predict, ';'-separated</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Birth cohort      reference cohort index for the oldest age in the span</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Youngest age      youngest age to predict</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Oldest age        oldest age to predict</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Dose              optional; leave blank to default to the final dose</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Label             optional; free-text label echoed into the results</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A Location-only row (cohort/ages/dose left blank) inherits those from the row above it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Check with: imurun -h yourfile.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Fit with:   imurun yourfile.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Address workbook output review feedback
</commit_message>
<xml_diff>
--- a/inst/extdata/imurun_example.xlsx
+++ b/inst/extdata/imurun_example.xlsx
@@ -7,9 +7,10 @@
   </bookViews>
   <sheets>
     <sheet name="instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="observations" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="locations" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="target" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="configuration" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="observations" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="locations" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="target" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -385,7 +386,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:A45"/>
+  <dimension ref="A1:A54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="100.711"/>
@@ -436,273 +437,336 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3. Save the file, then check it:   imurun -h yourfile.xlsx</t>
+          <t xml:space="preserve">  3. Review the configuration sheet, then save the file.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  4. Fix anything it flags, then fit: imurun yourfile.xlsx</t>
+          <t xml:space="preserve">  4. From R, check it: imurun::run_fit(c('-h', 'yourfile.xlsx'))</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  A bad edit fails the check with a clear message -- it cannot silently produce a wrong result.</t>
+          <t xml:space="preserve">  5. Fix anything it flags, then fit: imurun::run_fit('yourfile.xlsx')</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t xml:space="preserve">  A bad edit fails the check with a clear message -- it cannot silently produce a wrong result.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>This 'instructions' sheet is optional: imurun reads only the data sheets by name, so you may</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>delete it. Do not add a populations sheet or an observation-id column -- imurun handles both</t>
+          <t>This 'instructions' sheet is optional: imurun reads only the data sheets by name, so you may</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>for you. Extra columns you add for your own notes are ignored.</t>
+          <t>delete it. Do not add a populations sheet or an observation-id column -- imurun handles both</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t>for you. Extra columns you add for your own notes are ignored.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>observations sheet -- one row per sampled count:</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Location          the location of this count (must match a Location in the locations sheet)</t>
+          <t>configuration sheet -- sampler settings used for the fit:</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Reference cohort  positive whole-number cohort index, for the OLDEST age in the row</t>
+          <t xml:space="preserve">  iter              total iterations per chain (default 2000)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Youngest age      youngest age this count covers</t>
+          <t xml:space="preserve">  chains            number of chains (default 4)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Oldest age        oldest age this count covers (put the same age in both for a single age)</t>
+          <t xml:space="preserve">  seed              optional random seed for reproducibility</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Dose              which dose this count is for: 1 or 2</t>
+          <t xml:space="preserve">  warmup            optional warmup iterations per chain</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Vaccinated        how many were found vaccinated</t>
+          <t xml:space="preserve">  Leave seed/warmup blank to use the model defaults.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sampled           how many were sampled (Vaccinated must be &lt;= Sampled)</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Censored          optional; leave blank, or put 1 for a right-censored observation</t>
+          <t>observations sheet -- one row per sampled count:</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  A count covering several ages is split evenly across them, and the cohort of each younger</t>
+          <t xml:space="preserve">  Location          the location of this count (must match a Location in the locations sheet)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  age is stepped up so that age + cohort stays constant (a snapshot in time). If you prefer,</t>
+          <t xml:space="preserve">  Reference cohort  positive whole-number cohort index, for the OLDEST age in the row</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  you may use a single 'Age' column instead of the two age columns.</t>
+          <t xml:space="preserve">  Youngest age      youngest age this count covers</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t xml:space="preserve">  Oldest age        oldest age this count covers (put the same age in both for a single age)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>locations sheet -- your location hierarchy, written as a tree:</t>
+          <t xml:space="preserve">  Dose              which dose this count is for: 1 or 2</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Location          a unique name for the location (you choose the names)</t>
+          <t xml:space="preserve">  Vaccinated        how many were found vaccinated</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Parent location   the name of this location's parent (must be another Location in this sheet)</t>
+          <t xml:space="preserve">  Sampled           how many were sampled (Vaccinated must be &lt;= Sampled)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  IMPORTANT: there must be exactly ONE root -- the single top location whose Parent location</t>
+          <t xml:space="preserve">  Censored          optional; leave blank, or put 1 for a right-censored observation</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  is left BLANK. Every other location must name its parent, and the parents must chain up to</t>
+          <t xml:space="preserve">  A count covering several ages is split evenly across them, and the cohort of each younger</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  that one root (no loops, no second root). This is the most common thing to get wrong.</t>
+          <t xml:space="preserve">  age is stepped up so that age + cohort stays constant (a snapshot in time). If you prefer,</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t xml:space="preserve">  you may use a single 'Age' column instead of the two age columns.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>target sheet -- the populations to predict coverage for (required):</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Location          one or more locations to predict, ';'-separated</t>
+          <t>locations sheet -- your location hierarchy, written as a tree:</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Reference cohort  cohort index for the oldest age in the span</t>
+          <t xml:space="preserve">  Location          a unique name for the location (you choose the names)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Youngest age      youngest age to predict</t>
+          <t xml:space="preserve">  Parent location   the name of this location's parent (must be another Location in this sheet)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Oldest age        oldest age to predict</t>
+          <t xml:space="preserve">  IMPORTANT: there must be exactly ONE root -- the single top location whose Parent location</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Dose              optional; leave blank to default to the final dose</t>
+          <t xml:space="preserve">  is left BLANK. Every other location must name its parent, and the parents must chain up to</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Label             optional; free-text label echoed into the results</t>
+          <t xml:space="preserve">  that one root (no loops, no second root). This is the most common thing to get wrong.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  A Location-only row (cohort/ages/dose left blank) inherits those from the row above it.</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t>target sheet -- the populations to predict coverage for (required):</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Check with: imurun -h yourfile.xlsx</t>
+          <t xml:space="preserve">  Location          one or more locations to predict, ';'-separated</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Fit with:   imurun yourfile.xlsx</t>
+          <t xml:space="preserve">  Reference cohort  cohort index for the oldest age in the span</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Youngest age      youngest age to predict</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Oldest age        oldest age to predict</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Dose              optional; leave blank to default to the final dose</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Label             optional; free-text label echoed into the results</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A Location-only row (cohort/ages/dose left blank) inherits those from the row above it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Check from R: imurun::run_fit(c('-h', 'yourfile.xlsx'))</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Fit from R:   imurun::run_fit('yourfile.xlsx')</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>If you installed the optional command wrapper, 'imurun yourfile.xlsx' also works.</t>
         </is>
       </c>
     </row>
@@ -714,6 +778,109 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="7.711"/>
+    <col min="2" max="2" bestFit="1" customWidth="1" hidden="false" width="5.711"/>
+    <col min="3" max="3" bestFit="1" customWidth="1" hidden="false" width="40.711"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>iter</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Total iterations per chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>chains</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Number of chains</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Optional random seed for reproducibility</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>warmup</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Optional warmup iterations per chain</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C1"/>
+  <printOptions gridLines="1" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:G699"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -18227,7 +18394,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -18590,7 +18757,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>